<commit_message>
Sync journal indexing update (JRME)
Re-synced journal_indexing.xlsx from the updated Journal Profiles master:
JRME Scopus detail simplified to "Yes — Q1" and the "Highest SJR in the set"
note removed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/journal_indexing.xlsx
+++ b/data/xlsx/journal_indexing.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Yes — Q1 (SJR 1.40)</t>
+          <t>Yes — Q1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -583,11 +583,6 @@
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Highest SJR in the set</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>